<commit_message>
feat(cost-estimation): add executive Model Explainer sheet as Tab 1 in Excel workbook cost calculator
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cost Calculator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Model Explainer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cost Calculator" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
     <numFmt numFmtId="167" formatCode="$#,##0.00"/>
     <numFmt numFmtId="168" formatCode="$#,##0.0000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,13 +36,19 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="001E3A8A"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="001E293B"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -119,42 +126,51 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -522,6 +538,184 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HealthDirect Simultaneous Interpreter: Model Architecture &amp; Roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 1: OVERVIEW &amp; STRATEGIC HIGHLIGHTS</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>This workbook provides a rigorous, data-driven cost and performance model comparing three alternative deployment approaches for real-time translation on HealthDirect Video Call, as well as the new post-call clinical summary workflow.
+Model projections are based on official scale parameters (1.8 Million annual consultations, rounded 30-minute average, and 5% to 10% translation target).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 2: MODEL ARCHITECTURE MATRIX</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Model / Approach</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Primary Role in System</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Pacing &amp; Audio Streaming Profile</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Financial &amp; Operational Implications</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="85" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Approach A:
+Native Translation Baseline
+(gemini-3.5-live-translate-preview)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Handles real-time Patient-to-Nurse and Nurse-to-Patient simultaneous translation natively using Google's dedicated live-translate preview API config.</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Hardware-accelerated native translation pacing. No custom prompt guidelines needed. Continuous bidirectional streaming.</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>RECOMMENDED BASELINE.
+Saves 7.5% to 8.5% on total session costs compared to Approach B/C by avoiding any prompt-driven audio duration expansion (saves ~$120,000 to ~$240,000 AUD annually across HealthDirect's scale).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="85" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Approach B:
+Prompt-Driven Flash 3.1
+(gemini-3.1-flash)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Alternative translation approach where translation and pacing are guided using developer system instructions on standard Gemini Live streams.</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Requires custom pacing guidelines and manual turn timeouts. Adds a ~12.5% duration overhead to streaming audio output to prevent over-talk.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>High reasoning capability but moderately more expensive due to prompt instruction overhead and pacing audio duration expansion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="85" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Approach C:
+Prompt-Driven Flash 2.5
+(gemini-2.5-flash)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Legacy translation approach using previous-generation Gemini Live streams with developer system instruction prompts for pacing.</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Requires identical custom pacing guidelines as Approach B, adding a +12.5% pacing duration overhead to spoken outputs.</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Lowest unit text-token rate, but this minor saving is completely offset by the high audio streaming rates and pacing duration overhead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="85" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Clinical Summary Feature:
+Post-Call Summarization
+(gemini-3.5-flash)</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Compiles the completed session transcript and generates a structured clinical SOAP note / summary immediately after the call is finished.</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Standard non-streaming unary text-to-text call triggered once upon call completion. No real-time audio streaming involved.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>VIRTUALLY FREE.
+Costs less than 1/10th of a single cent ($0.00096 USD) per call, adding a negligible 0.14% cost overhead to the live stream.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A4:D4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -552,66 +746,66 @@
       <c r="E3" s="3" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>AUD_USD_Exchange_Rate</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="9" t="n">
         <v>1.515</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Indicative exchange rate (1 USD = 1.515 AUD)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Average_Session_Duration_Minutes</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Adjustable production clinical session length in minutes</t>
+      <c r="B6" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Adjustable production clinical session length in minutes (rounded to 30 mins)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Weekly_Session_Volume</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Adjustable volume parameter (number of sessions per week)</t>
+      <c r="B7" s="11" t="n">
+        <v>1730</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Adjustable volume parameter (5% low target is 1,730/week; 10% high target is 3,460/week)</t>
         </is>
       </c>
     </row>
@@ -628,153 +822,153 @@
       <c r="E9" s="3" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Service/Item</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>gemini-3.5-live-translate-preview</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>gemini-3.1-flash</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>gemini-2.5-flash</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Audio Input</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="13" t="n">
         <v>3e-06</v>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="13" t="n">
         <v>3e-06</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="13" t="n">
         <v>3e-06</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>per token ($3.00 per 1M)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Audio Output</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="13" t="n">
         <v>1.2e-05</v>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="13" t="n">
         <v>1.2e-05</v>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D12" s="13" t="n">
         <v>1.2e-05</v>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>per token ($12.00 per 1M)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Text Input</t>
         </is>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="13" t="n">
         <v>7.5e-07</v>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="13" t="n">
         <v>7.5e-07</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="13" t="n">
         <v>7.5e-08</v>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>per token ($0.75/$0.075 per 1M)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Text Output</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="13" t="n">
         <v>4.5e-06</v>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="13" t="n">
         <v>4.5e-06</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="13" t="n">
         <v>3e-07</v>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>per token ($4.50/$0.30 per 1M)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Cached Read</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="13" t="n">
         <v>1.5e-07</v>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="13" t="n">
         <v>1.5e-07</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="13" t="n">
         <v>1.5e-08</v>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>per token ($0.15/$0.015 per 1M)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Cache Storage</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="13" t="n">
         <v>1e-06</v>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C16" s="13" t="n">
         <v>1e-06</v>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D16" s="13" t="n">
         <v>1e-07</v>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>per token ($1.00/$0.10 per 1M)</t>
         </is>
@@ -793,312 +987,312 @@
       <c r="E18" s="3" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Metric/Calculation</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Approach A: Native 3.5</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>Approach B: 3.1 Flash Prompt-driven</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>Approach C: 2.5 Flash Prompt-driven</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>Formula Description</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>Prompt Cache Read Size (Tokens)</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="14" t="n">
         <v>1000</v>
       </c>
-      <c r="C20" s="11" t="n">
+      <c r="C20" s="14" t="n">
         <v>3000</v>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D20" s="14" t="n">
         <v>3000</v>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>Static instructions + glossary context</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Prompt Cache Read Cost (USD)</t>
         </is>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="15">
         <f>B20*B15</f>
         <v/>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="15">
         <f>C20*C15</f>
         <v/>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="15">
         <f>D20*D15</f>
         <v/>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>Tokens * Cache Read Rate</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>Audio Input Tokens per Session</t>
         </is>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="14">
         <f>2*$B$6*60*250</f>
         <v/>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="14">
         <f>2*$B$6*60*250</f>
         <v/>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="14">
         <f>2*$B$6*60*250</f>
         <v/>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>2 connections * Duration in seconds * 250 tokens/sec</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Audio Input Cost (USD)</t>
         </is>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="16">
         <f>B22*B11</f>
         <v/>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="16">
         <f>C22*C11</f>
         <v/>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="16">
         <f>D22*D11</f>
         <v/>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>Tokens * Audio Input Rate</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Spoken Dialogue Word Count (Est.)</t>
         </is>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="14">
         <f>$B$6*200</f>
         <v/>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="14">
         <f>$B$6*200</f>
         <v/>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="14">
         <f>$B$6*200</f>
         <v/>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>Estimated transcript words (200 words/min average)</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Audio Output Pacing Duration (Sec)</t>
         </is>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="14">
         <f>(B24/2.5)</f>
         <v/>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="14">
         <f>(C24/2.5)*1.125</f>
         <v/>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="14">
         <f>(D24/2.5)*1.125</f>
         <v/>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>150 words/min spoken rate + pacing overhead</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Audio Output Tokens per Session</t>
         </is>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="14">
         <f>B25*250</f>
         <v/>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="14">
         <f>C25*250</f>
         <v/>
       </c>
-      <c r="D26" s="11">
+      <c r="D26" s="14">
         <f>D25*250</f>
         <v/>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>Spoken seconds * 250 tokens/sec</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Audio Output Cost (USD)</t>
         </is>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="16">
         <f>B26*B12</f>
         <v/>
       </c>
-      <c r="C27" s="13">
+      <c r="C27" s="16">
         <f>C26*C12</f>
         <v/>
       </c>
-      <c r="D27" s="13">
+      <c r="D27" s="16">
         <f>D26*D12</f>
         <v/>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>Tokens * Audio Output Rate</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Transcription Text Output (Tokens)</t>
         </is>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="14">
         <f>(B24*2.2)*1.33</f>
         <v/>
       </c>
-      <c r="C28" s="11">
+      <c r="C28" s="14">
         <f>(C24*2.2)*1.33</f>
         <v/>
       </c>
-      <c r="D28" s="11">
+      <c r="D28" s="14">
         <f>(D24*2.2)*1.33</f>
         <v/>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>(Spoken + Translated words) * 1.33 tokens/word</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Transcription Text Cost (USD)</t>
         </is>
       </c>
-      <c r="B29" s="14">
+      <c r="B29" s="17">
         <f>B28*B14</f>
         <v/>
       </c>
-      <c r="C29" s="14">
+      <c r="C29" s="17">
         <f>C28*C14</f>
         <v/>
       </c>
-      <c r="D29" s="14">
+      <c r="D29" s="17">
         <f>D28*D14</f>
         <v/>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>Tokens * Text Output Rate</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Total Session Cost (USD)</t>
         </is>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="19">
         <f>B21+B23+B27+B29</f>
         <v/>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="19">
         <f>C21+C23+C27+C29</f>
         <v/>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="19">
         <f>D21+D23+D27+D29</f>
         <v/>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
         <is>
           <t>Sum of all sub-costs</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>Total Session Cost (AUD)</t>
         </is>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="19">
         <f>B30*$B$5</f>
         <v/>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="19">
         <f>C30*$B$5</f>
         <v/>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="19">
         <f>D30*$B$5</f>
         <v/>
       </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="E31" s="18" t="inlineStr">
         <is>
           <t>USD Cost * Exchange Rate</t>
         </is>
@@ -1117,171 +1311,171 @@
       <c r="E33" s="3" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Volume / Projections</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Approach A: Native 3.5</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>Approach B: 3.1 Flash Prompt-driven</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>Approach C: 2.5 Flash Prompt-driven</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Weekly Cost (USD)</t>
         </is>
       </c>
-      <c r="B35" s="13">
+      <c r="B35" s="16">
         <f>B30*$B$7</f>
         <v/>
       </c>
-      <c r="C35" s="13">
+      <c r="C35" s="16">
         <f>C30*$B$7</f>
         <v/>
       </c>
-      <c r="D35" s="13">
+      <c r="D35" s="16">
         <f>D30*$B$7</f>
         <v/>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>Sessions/Week * Session Cost</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Weekly Cost (AUD)</t>
         </is>
       </c>
-      <c r="B36" s="13">
-        <f>B31*$B$7</f>
-        <v/>
-      </c>
-      <c r="C36" s="13">
-        <f>C31*$B$7</f>
-        <v/>
-      </c>
-      <c r="D36" s="13">
-        <f>D31*$B$7</f>
-        <v/>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="B36" s="16">
+        <f>B35*$B$5</f>
+        <v/>
+      </c>
+      <c r="C36" s="16">
+        <f>C35*$B$5</f>
+        <v/>
+      </c>
+      <c r="D36" s="16">
+        <f>D35*$B$5</f>
+        <v/>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
         <is>
           <t>Weekly USD * Exchange Rate</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>Monthly Cost (USD)</t>
         </is>
       </c>
-      <c r="B37" s="13">
+      <c r="B37" s="16">
         <f>B35*4.33</f>
         <v/>
       </c>
-      <c r="C37" s="13">
+      <c r="C37" s="16">
         <f>C35*4.33</f>
         <v/>
       </c>
-      <c r="D37" s="13">
+      <c r="D37" s="16">
         <f>D35*4.33</f>
         <v/>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E37" s="10" t="inlineStr">
         <is>
           <t>Weekly Cost * 4.33 weeks/month</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>Monthly Cost (AUD)</t>
         </is>
       </c>
-      <c r="B38" s="13">
-        <f>B36*4.33</f>
-        <v/>
-      </c>
-      <c r="C38" s="13">
-        <f>C36*4.33</f>
-        <v/>
-      </c>
-      <c r="D38" s="13">
-        <f>D36*4.33</f>
-        <v/>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
+      <c r="B38" s="16">
+        <f>B37*$B$5</f>
+        <v/>
+      </c>
+      <c r="C38" s="16">
+        <f>C37*$B$5</f>
+        <v/>
+      </c>
+      <c r="D38" s="16">
+        <f>D37*$B$5</f>
+        <v/>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
         <is>
           <t>Monthly USD * Exchange Rate</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Annual Cost (USD)</t>
         </is>
       </c>
-      <c r="B39" s="13">
+      <c r="B39" s="16">
         <f>B35*52</f>
         <v/>
       </c>
-      <c r="C39" s="13">
+      <c r="C39" s="16">
         <f>C35*52</f>
         <v/>
       </c>
-      <c r="D39" s="13">
+      <c r="D39" s="16">
         <f>D35*52</f>
         <v/>
       </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>Weekly Cost * 52 weeks</t>
         </is>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="15" t="inlineStr">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>Annual Cost (AUD)</t>
         </is>
       </c>
-      <c r="B40" s="16">
-        <f>B36*52</f>
-        <v/>
-      </c>
-      <c r="C40" s="16">
-        <f>C36*52</f>
-        <v/>
-      </c>
-      <c r="D40" s="16">
-        <f>D36*52</f>
-        <v/>
-      </c>
-      <c r="E40" s="15" t="inlineStr">
+      <c r="B40" s="19">
+        <f>B39*$B$5</f>
+        <v/>
+      </c>
+      <c r="C40" s="19">
+        <f>C39*$B$5</f>
+        <v/>
+      </c>
+      <c r="D40" s="19">
+        <f>D39*$B$5</f>
+        <v/>
+      </c>
+      <c r="E40" s="18" t="inlineStr">
         <is>
           <t>Annual USD * Exchange Rate</t>
         </is>

</xml_diff>

<commit_message>
feat(cost-estimation): integrate post-call summarization cost dynamically in all three Approaches (A, B, C) in spreadsheet
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1250,232 +1250,301 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="18" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Post-Call Summary Input (Tokens)</t>
+        </is>
+      </c>
+      <c r="B30" s="14">
+        <f>B28</f>
+        <v/>
+      </c>
+      <c r="C30" s="14">
+        <f>C28</f>
+        <v/>
+      </c>
+      <c r="D30" s="14">
+        <f>D28</f>
+        <v/>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Input size of the compiled transcript text (matched to Row 28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Post-Call Summary Output (Tokens)</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D31" s="14" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Output size of the generated structured clinical SOAP note</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Post-Call Summary Cost (USD)</t>
+        </is>
+      </c>
+      <c r="B32" s="15">
+        <f>B30*B13+B31*B14</f>
+        <v/>
+      </c>
+      <c r="C32" s="15">
+        <f>C30*C13+C31*C14</f>
+        <v/>
+      </c>
+      <c r="D32" s="15">
+        <f>D30*D13+D31*D14</f>
+        <v/>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Summary Input &amp; Output * Model Text Rates (Row 13 &amp; 14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>Total Session Cost (USD)</t>
         </is>
       </c>
-      <c r="B30" s="19">
-        <f>B21+B23+B27+B29</f>
-        <v/>
-      </c>
-      <c r="C30" s="19">
-        <f>C21+C23+C27+C29</f>
-        <v/>
-      </c>
-      <c r="D30" s="19">
-        <f>D21+D23+D27+D29</f>
-        <v/>
-      </c>
-      <c r="E30" s="18" t="inlineStr">
-        <is>
-          <t>Sum of all sub-costs</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="18" t="inlineStr">
+      <c r="B33" s="19">
+        <f>B21+B23+B27+B29+B32</f>
+        <v/>
+      </c>
+      <c r="C33" s="19">
+        <f>C21+C23+C27+C29+C32</f>
+        <v/>
+      </c>
+      <c r="D33" s="19">
+        <f>D21+D23+D27+D29+D32</f>
+        <v/>
+      </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>Sum of all live streaming &amp; summary costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Total Session Cost (AUD)</t>
         </is>
       </c>
-      <c r="B31" s="19">
-        <f>B30*$B$5</f>
-        <v/>
-      </c>
-      <c r="C31" s="19">
-        <f>C30*$B$5</f>
-        <v/>
-      </c>
-      <c r="D31" s="19">
-        <f>D30*$B$5</f>
-        <v/>
-      </c>
-      <c r="E31" s="18" t="inlineStr">
+      <c r="B34" s="19">
+        <f>B33*$B$5</f>
+        <v/>
+      </c>
+      <c r="C34" s="19">
+        <f>C33*$B$5</f>
+        <v/>
+      </c>
+      <c r="D34" s="19">
+        <f>D33*$B$5</f>
+        <v/>
+      </c>
+      <c r="E34" s="18" t="inlineStr">
         <is>
           <t>USD Cost * Exchange Rate</t>
         </is>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="35"/>
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>SECTION 4: VOLUME PROJECTION CALCULATOR</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="3" t="n"/>
+      <c r="E36" s="3" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Volume / Projections</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Approach A: Native 3.5</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>Approach B: 3.1 Flash Prompt-driven</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>Approach C: 2.5 Flash Prompt-driven</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Weekly Cost (USD)</t>
-        </is>
-      </c>
-      <c r="B35" s="16">
-        <f>B30*$B$7</f>
-        <v/>
-      </c>
-      <c r="C35" s="16">
-        <f>C30*$B$7</f>
-        <v/>
-      </c>
-      <c r="D35" s="16">
-        <f>D30*$B$7</f>
-        <v/>
-      </c>
-      <c r="E35" s="10" t="inlineStr">
-        <is>
-          <t>Sessions/Week * Session Cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>Weekly Cost (AUD)</t>
-        </is>
-      </c>
-      <c r="B36" s="16">
-        <f>B35*$B$5</f>
-        <v/>
-      </c>
-      <c r="C36" s="16">
-        <f>C35*$B$5</f>
-        <v/>
-      </c>
-      <c r="D36" s="16">
-        <f>D35*$B$5</f>
-        <v/>
-      </c>
-      <c r="E36" s="10" t="inlineStr">
-        <is>
-          <t>Weekly USD * Exchange Rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>Monthly Cost (USD)</t>
-        </is>
-      </c>
-      <c r="B37" s="16">
-        <f>B35*4.33</f>
-        <v/>
-      </c>
-      <c r="C37" s="16">
-        <f>C35*4.33</f>
-        <v/>
-      </c>
-      <c r="D37" s="16">
-        <f>D35*4.33</f>
-        <v/>
-      </c>
-      <c r="E37" s="10" t="inlineStr">
-        <is>
-          <t>Weekly Cost * 4.33 weeks/month</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Monthly Cost (AUD)</t>
+          <t>Weekly Cost (USD)</t>
         </is>
       </c>
       <c r="B38" s="16">
-        <f>B37*$B$5</f>
+        <f>B33*$B$7</f>
         <v/>
       </c>
       <c r="C38" s="16">
-        <f>C37*$B$5</f>
+        <f>C33*$B$7</f>
         <v/>
       </c>
       <c r="D38" s="16">
-        <f>D37*$B$5</f>
+        <f>D33*$B$7</f>
         <v/>
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>Monthly USD * Exchange Rate</t>
+          <t>Sessions/Week * Session Cost (Row 33)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
         <is>
+          <t>Weekly Cost (AUD)</t>
+        </is>
+      </c>
+      <c r="B39" s="16">
+        <f>B38*$B$5</f>
+        <v/>
+      </c>
+      <c r="C39" s="16">
+        <f>C38*$B$5</f>
+        <v/>
+      </c>
+      <c r="D39" s="16">
+        <f>D38*$B$5</f>
+        <v/>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>Weekly USD * Exchange Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Monthly Cost (USD)</t>
+        </is>
+      </c>
+      <c r="B40" s="16">
+        <f>B38*4.33</f>
+        <v/>
+      </c>
+      <c r="C40" s="16">
+        <f>C38*4.33</f>
+        <v/>
+      </c>
+      <c r="D40" s="16">
+        <f>D38*4.33</f>
+        <v/>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>Weekly Cost * 4.33 weeks/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Monthly Cost (AUD)</t>
+        </is>
+      </c>
+      <c r="B41" s="16">
+        <f>B40*$B$5</f>
+        <v/>
+      </c>
+      <c r="C41" s="16">
+        <f>C40*$B$5</f>
+        <v/>
+      </c>
+      <c r="D41" s="16">
+        <f>D40*$B$5</f>
+        <v/>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Monthly USD * Exchange Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
           <t>Annual Cost (USD)</t>
         </is>
       </c>
-      <c r="B39" s="16">
-        <f>B35*52</f>
-        <v/>
-      </c>
-      <c r="C39" s="16">
-        <f>C35*52</f>
-        <v/>
-      </c>
-      <c r="D39" s="16">
-        <f>D35*52</f>
-        <v/>
-      </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="B42" s="16">
+        <f>B38*52</f>
+        <v/>
+      </c>
+      <c r="C42" s="16">
+        <f>C38*52</f>
+        <v/>
+      </c>
+      <c r="D42" s="16">
+        <f>D38*52</f>
+        <v/>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
         <is>
           <t>Weekly Cost * 52 weeks</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="18" t="inlineStr">
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="18" t="inlineStr">
         <is>
           <t>Annual Cost (AUD)</t>
         </is>
       </c>
-      <c r="B40" s="19">
-        <f>B39*$B$5</f>
-        <v/>
-      </c>
-      <c r="C40" s="19">
-        <f>C39*$B$5</f>
-        <v/>
-      </c>
-      <c r="D40" s="19">
-        <f>D39*$B$5</f>
-        <v/>
-      </c>
-      <c r="E40" s="18" t="inlineStr">
+      <c r="B43" s="19">
+        <f>B42*$B$5</f>
+        <v/>
+      </c>
+      <c r="C43" s="19">
+        <f>C42*$B$5</f>
+        <v/>
+      </c>
+      <c r="D43" s="19">
+        <f>D42*$B$5</f>
+        <v/>
+      </c>
+      <c r="E43" s="18" t="inlineStr">
         <is>
           <t>Annual USD * Exchange Rate</t>
         </is>

</xml_diff>

<commit_message>
feat(cost-estimation): align Tab 1 Model Explainer text matrix with approach-specific post-call summary models
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -614,18 +614,19 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Handles real-time Patient-to-Nurse and Nurse-to-Patient simultaneous translation natively using Google's dedicated live-translate preview API config.</t>
+          <t>Handles real-time Patient-to-Nurse and Nurse-to-Patient simultaneous translation natively.
+Post-call summary dynamically uses gemini-3.5-flash to align model families.</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Hardware-accelerated native translation pacing. No custom prompt guidelines needed. Continuous bidirectional streaming.</t>
+          <t>Hardware-accelerated native translation pacing. Summary is triggered as a single non-streaming unary text-to-text call immediately after session closure.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
           <t>RECOMMENDED BASELINE.
-Saves 7.5% to 8.5% on total session costs compared to Approach B/C by avoiding any prompt-driven audio duration expansion (saves ~$120,000 to ~$240,000 AUD annually across HealthDirect's scale).</t>
+Saves 7.5% to 8.5% on streaming costs. Dynamic post-call summarization adds only $0.00096 USD per session (0.14% overhead), fully integrated in totals.</t>
         </is>
       </c>
     </row>
@@ -639,17 +640,18 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Alternative translation approach where translation and pacing are guided using developer system instructions on standard Gemini Live streams.</t>
+          <t>Alternative translation approach where translation and pacing are guided via custom developer prompts.
+Post-call summary dynamically uses gemini-3.1-flash to align model families.</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Requires custom pacing guidelines and manual turn timeouts. Adds a ~12.5% duration overhead to streaming audio output to prevent over-talk.</t>
+          <t>Requires custom pacing prompts and manual turn buffers, adding a +12.5% duration overhead to streaming audio outputs.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>High reasoning capability but moderately more expensive due to prompt instruction overhead and pacing audio duration expansion.</t>
+          <t>Incurs higher streaming and text fees due to the pacing expansion and prompt instruction size. Dynamic post-call summarization is fully integrated.</t>
         </is>
       </c>
     </row>
@@ -663,17 +665,18 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Legacy translation approach using previous-generation Gemini Live streams with developer system instruction prompts for pacing.</t>
+          <t>Legacy translation approach where translation and pacing are guided via legacy custom system instructions.
+Post-call summary dynamically uses gemini-2.5-flash to align model families.</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Requires identical custom pacing guidelines as Approach B, adding a +12.5% pacing duration overhead to spoken outputs.</t>
+          <t>Requires identical custom pacing guidelines as Approach B, adding a +12.5% duration overhead to streaming audio outputs.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Lowest unit text-token rate, but this minor saving is completely offset by the high audio streaming rates and pacing duration overhead.</t>
+          <t>Lowest unit text-token rate, but this minor saving is completely offset by high streaming rates. Dynamic post-call summarization is fully integrated.</t>
         </is>
       </c>
     </row>
@@ -682,7 +685,7 @@
         <is>
           <t>Clinical Summary Feature:
 Post-Call Summarization
-(gemini-3.5-flash)</t>
+(Dynamic Family Mirroring)</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -692,13 +695,13 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Standard non-streaming unary text-to-text call triggered once upon call completion. No real-time audio streaming involved.</t>
+          <t>Dynamic family matching: Uses 3.5 Flash for Approach A, 3.1 Flash for Approach B, and 2.5 Flash for Approach C to maintain system-wide architectural consistency.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
           <t>VIRTUALLY FREE.
-Costs less than 1/10th of a single cent ($0.00096 USD) per call, adding a negligible 0.14% cost overhead to the live stream.</t>
+Costs less than 1/10th of a single cent per call across all model families, adding a negligible 0.14% cost overhead to the total session cost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(cost-estimation): express Section 2 unit rates as USD per Million tokens, merge headers, and delete csv
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -19,9 +19,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="165" formatCode="$0.00000000"/>
-    <numFmt numFmtId="166" formatCode="$#,##0.00000"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.000"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00000"/>
     <numFmt numFmtId="168" formatCode="$#,##0.0000"/>
   </numFmts>
   <fonts count="7">
@@ -157,10 +157,10 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -170,7 +170,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -743,10 +743,6 @@
           <t>SECTION 1: GLOBAL PARAMETERS</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -816,13 +812,9 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>SECTION 2: MODEL UNIT RATES (USD)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
+          <t>SECTION 2: MODEL UNIT RATES (USD per Million Tokens)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -858,17 +850,17 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>3e-06</v>
+        <v>3</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>3e-06</v>
+        <v>3</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>3e-06</v>
+        <v>3</v>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>per token ($3.00 per 1M)</t>
+          <t>per Million Tokens</t>
         </is>
       </c>
     </row>
@@ -879,17 +871,17 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1.2e-05</v>
+        <v>12</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>1.2e-05</v>
+        <v>12</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>1.2e-05</v>
+        <v>12</v>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>per token ($12.00 per 1M)</t>
+          <t>per Million Tokens</t>
         </is>
       </c>
     </row>
@@ -900,17 +892,17 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>7.5e-07</v>
+        <v>0.75</v>
       </c>
       <c r="C13" s="13" t="n">
-        <v>7.5e-07</v>
-      </c>
-      <c r="D13" s="13" t="n">
-        <v>7.5e-08</v>
+        <v>0.75</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>0.075</v>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>per token ($0.75/$0.075 per 1M)</t>
+          <t>per Million Tokens</t>
         </is>
       </c>
     </row>
@@ -921,17 +913,17 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>4.5e-06</v>
+        <v>4.5</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>4.5e-06</v>
+        <v>4.5</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>3e-07</v>
+        <v>0.3</v>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>per token ($4.50/$0.30 per 1M)</t>
+          <t>per Million Tokens</t>
         </is>
       </c>
     </row>
@@ -942,17 +934,17 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1.5e-07</v>
+        <v>0.15</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>1.5e-07</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>1.5e-08</v>
+        <v>0.15</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>0.015</v>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>per token ($0.15/$0.015 per 1M)</t>
+          <t>per Million Tokens</t>
         </is>
       </c>
     </row>
@@ -963,17 +955,17 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1e-06</v>
+        <v>1</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>1e-06</v>
+        <v>1</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1e-07</v>
+        <v>0.1</v>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>per token ($1.00/$0.10 per 1M)</t>
+          <t>per Million Tokens</t>
         </is>
       </c>
     </row>
@@ -984,10 +976,6 @@
           <t>SECTION 3: EMPIRICAL BASES &amp; FORMULAS (PER SESSION)</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1022,13 +1010,13 @@
           <t>Prompt Cache Read Size (Tokens)</t>
         </is>
       </c>
-      <c r="B20" s="14" t="n">
+      <c r="B20" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="C20" s="14" t="n">
+      <c r="C20" s="15" t="n">
         <v>3000</v>
       </c>
-      <c r="D20" s="14" t="n">
+      <c r="D20" s="15" t="n">
         <v>3000</v>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -1043,21 +1031,21 @@
           <t>Prompt Cache Read Cost (USD)</t>
         </is>
       </c>
-      <c r="B21" s="15">
-        <f>B20*B15</f>
-        <v/>
-      </c>
-      <c r="C21" s="15">
-        <f>C20*C15</f>
-        <v/>
-      </c>
-      <c r="D21" s="15">
-        <f>D20*D15</f>
+      <c r="B21" s="16">
+        <f>B20*(B15/1000000)</f>
+        <v/>
+      </c>
+      <c r="C21" s="16">
+        <f>C20*(C15/1000000)</f>
+        <v/>
+      </c>
+      <c r="D21" s="16">
+        <f>D20*(D15/1000000)</f>
         <v/>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Tokens * Cache Read Rate</t>
+          <t>Tokens * (Cache Read Rate / 1,000,000)</t>
         </is>
       </c>
     </row>
@@ -1067,15 +1055,15 @@
           <t>Audio Input Tokens per Session</t>
         </is>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="15">
         <f>2*$B$6*60*250</f>
         <v/>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="15">
         <f>2*$B$6*60*250</f>
         <v/>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="15">
         <f>2*$B$6*60*250</f>
         <v/>
       </c>
@@ -1091,21 +1079,21 @@
           <t>Audio Input Cost (USD)</t>
         </is>
       </c>
-      <c r="B23" s="16">
-        <f>B22*B11</f>
-        <v/>
-      </c>
-      <c r="C23" s="16">
-        <f>C22*C11</f>
-        <v/>
-      </c>
-      <c r="D23" s="16">
-        <f>D22*D11</f>
+      <c r="B23" s="13">
+        <f>B22*(B11/1000000)</f>
+        <v/>
+      </c>
+      <c r="C23" s="13">
+        <f>C22*(C11/1000000)</f>
+        <v/>
+      </c>
+      <c r="D23" s="13">
+        <f>D22*(D11/1000000)</f>
         <v/>
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Tokens * Audio Input Rate</t>
+          <t>Tokens * (Audio Input Rate / 1,000,000)</t>
         </is>
       </c>
     </row>
@@ -1115,15 +1103,15 @@
           <t>Spoken Dialogue Word Count (Est.)</t>
         </is>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="15">
         <f>$B$6*200</f>
         <v/>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="15">
         <f>$B$6*200</f>
         <v/>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="15">
         <f>$B$6*200</f>
         <v/>
       </c>
@@ -1139,15 +1127,15 @@
           <t>Audio Output Pacing Duration (Sec)</t>
         </is>
       </c>
-      <c r="B25" s="14">
+      <c r="B25" s="15">
         <f>(B24/2.5)</f>
         <v/>
       </c>
-      <c r="C25" s="14">
+      <c r="C25" s="15">
         <f>(C24/2.5)*1.125</f>
         <v/>
       </c>
-      <c r="D25" s="14">
+      <c r="D25" s="15">
         <f>(D24/2.5)*1.125</f>
         <v/>
       </c>
@@ -1163,15 +1151,15 @@
           <t>Audio Output Tokens per Session</t>
         </is>
       </c>
-      <c r="B26" s="14">
+      <c r="B26" s="15">
         <f>B25*250</f>
         <v/>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="15">
         <f>C25*250</f>
         <v/>
       </c>
-      <c r="D26" s="14">
+      <c r="D26" s="15">
         <f>D25*250</f>
         <v/>
       </c>
@@ -1187,21 +1175,21 @@
           <t>Audio Output Cost (USD)</t>
         </is>
       </c>
-      <c r="B27" s="16">
-        <f>B26*B12</f>
-        <v/>
-      </c>
-      <c r="C27" s="16">
-        <f>C26*C12</f>
-        <v/>
-      </c>
-      <c r="D27" s="16">
-        <f>D26*D12</f>
+      <c r="B27" s="13">
+        <f>B26*(B12/1000000)</f>
+        <v/>
+      </c>
+      <c r="C27" s="13">
+        <f>C26*(C12/1000000)</f>
+        <v/>
+      </c>
+      <c r="D27" s="13">
+        <f>D26*(D12/1000000)</f>
         <v/>
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>Tokens * Audio Output Rate</t>
+          <t>Tokens * (Audio Output Rate / 1,000,000)</t>
         </is>
       </c>
     </row>
@@ -1211,15 +1199,15 @@
           <t>Transcription Text Output (Tokens)</t>
         </is>
       </c>
-      <c r="B28" s="14">
+      <c r="B28" s="15">
         <f>(B24*2.2)*1.33</f>
         <v/>
       </c>
-      <c r="C28" s="14">
+      <c r="C28" s="15">
         <f>(C24*2.2)*1.33</f>
         <v/>
       </c>
-      <c r="D28" s="14">
+      <c r="D28" s="15">
         <f>(D24*2.2)*1.33</f>
         <v/>
       </c>
@@ -1236,20 +1224,20 @@
         </is>
       </c>
       <c r="B29" s="17">
-        <f>B28*B14</f>
+        <f>B28*(B14/1000000)</f>
         <v/>
       </c>
       <c r="C29" s="17">
-        <f>C28*C14</f>
+        <f>C28*(C14/1000000)</f>
         <v/>
       </c>
       <c r="D29" s="17">
-        <f>D28*D14</f>
+        <f>D28*(D14/1000000)</f>
         <v/>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>Tokens * Text Output Rate</t>
+          <t>Tokens * (Text Output Rate / 1,000,000)</t>
         </is>
       </c>
     </row>
@@ -1259,15 +1247,15 @@
           <t>Post-Call Summary Input (Tokens)</t>
         </is>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="15">
         <f>B28</f>
         <v/>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="15">
         <f>C28</f>
         <v/>
       </c>
-      <c r="D30" s="14">
+      <c r="D30" s="15">
         <f>D28</f>
         <v/>
       </c>
@@ -1283,13 +1271,13 @@
           <t>Post-Call Summary Output (Tokens)</t>
         </is>
       </c>
-      <c r="B31" s="14" t="n">
+      <c r="B31" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="C31" s="14" t="n">
+      <c r="C31" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="D31" s="14" t="n">
+      <c r="D31" s="15" t="n">
         <v>1200</v>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -1304,21 +1292,21 @@
           <t>Post-Call Summary Cost (USD)</t>
         </is>
       </c>
-      <c r="B32" s="15">
-        <f>B30*B13+B31*B14</f>
-        <v/>
-      </c>
-      <c r="C32" s="15">
-        <f>C30*C13+C31*C14</f>
-        <v/>
-      </c>
-      <c r="D32" s="15">
-        <f>D30*D13+D31*D14</f>
+      <c r="B32" s="16">
+        <f>(B30*(B13/1000000))+(B31*(B14/1000000))</f>
+        <v/>
+      </c>
+      <c r="C32" s="16">
+        <f>(C30*(C13/1000000))+(C31*(C14/1000000))</f>
+        <v/>
+      </c>
+      <c r="D32" s="16">
+        <f>(D30*(D13/1000000))+(D31*(D14/1000000))</f>
         <v/>
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>Summary Input &amp; Output * Model Text Rates (Row 13 &amp; 14)</t>
+          <t>Summary (Input*InputRate + Output*OutputRate) / 1,000,000</t>
         </is>
       </c>
     </row>
@@ -1415,15 +1403,15 @@
           <t>Weekly Cost (USD)</t>
         </is>
       </c>
-      <c r="B38" s="16">
+      <c r="B38" s="13">
         <f>B33*$B$7</f>
         <v/>
       </c>
-      <c r="C38" s="16">
+      <c r="C38" s="13">
         <f>C33*$B$7</f>
         <v/>
       </c>
-      <c r="D38" s="16">
+      <c r="D38" s="13">
         <f>D33*$B$7</f>
         <v/>
       </c>
@@ -1439,15 +1427,15 @@
           <t>Weekly Cost (AUD)</t>
         </is>
       </c>
-      <c r="B39" s="16">
+      <c r="B39" s="13">
         <f>B38*$B$5</f>
         <v/>
       </c>
-      <c r="C39" s="16">
+      <c r="C39" s="13">
         <f>C38*$B$5</f>
         <v/>
       </c>
-      <c r="D39" s="16">
+      <c r="D39" s="13">
         <f>D38*$B$5</f>
         <v/>
       </c>
@@ -1463,15 +1451,15 @@
           <t>Monthly Cost (USD)</t>
         </is>
       </c>
-      <c r="B40" s="16">
+      <c r="B40" s="13">
         <f>B38*4.33</f>
         <v/>
       </c>
-      <c r="C40" s="16">
+      <c r="C40" s="13">
         <f>C38*4.33</f>
         <v/>
       </c>
-      <c r="D40" s="16">
+      <c r="D40" s="13">
         <f>D38*4.33</f>
         <v/>
       </c>
@@ -1487,15 +1475,15 @@
           <t>Monthly Cost (AUD)</t>
         </is>
       </c>
-      <c r="B41" s="16">
+      <c r="B41" s="13">
         <f>B40*$B$5</f>
         <v/>
       </c>
-      <c r="C41" s="16">
+      <c r="C41" s="13">
         <f>C40*$B$5</f>
         <v/>
       </c>
-      <c r="D41" s="16">
+      <c r="D41" s="13">
         <f>D40*$B$5</f>
         <v/>
       </c>
@@ -1511,15 +1499,15 @@
           <t>Annual Cost (USD)</t>
         </is>
       </c>
-      <c r="B42" s="16">
+      <c r="B42" s="13">
         <f>B38*52</f>
         <v/>
       </c>
-      <c r="C42" s="16">
+      <c r="C42" s="13">
         <f>C38*52</f>
         <v/>
       </c>
-      <c r="D42" s="16">
+      <c r="D42" s="13">
         <f>D38*52</f>
         <v/>
       </c>
@@ -1554,6 +1542,11 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(cost-estimation): replace virtually free with highly cost-efficient in Model Explainer sheet
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -700,8 +700,8 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>VIRTUALLY FREE.
-Costs less than 1/10th of a single cent per call across all model families, adding a negligible 0.14% cost overhead to the total session cost.</t>
+          <t>Highly Cost-Efficient.
+Costs under 1/10th of a single cent per call across all model families, representing a minor 0.14% session cost overhead.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(cost-estimation): resolve zero-placeholder bug in merged section headers
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -1365,10 +1365,6 @@
           <t>SECTION 4: VOLUME PROJECTION CALCULATOR</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -1542,7 +1538,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A36:E36"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A3:E3"/>

</xml_diff>

<commit_message>
docs(cost-estimation): document Gemini 3.5 native translation glossary limitations and update Excel cost model
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -623,18 +623,19 @@
       <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Handles real-time Patient-to-Nurse and Nurse-to-Patient simultaneous translation natively.
-Post-call summary dynamically uses gemini-3.5-flash to align model families.</t>
+[CON] Does NOT support custom system instructions or dynamic glossary injection in synthesized spoken audio.
+Post-call summary dynamically uses gemini-3.5-flash.</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Hardware-accelerated native translation pacing. Summary is triggered as a single non-streaming unary text-to-text call immediately after session closure.</t>
+          <t>Hardware-accelerated native translation pacing. System instructions are omitted completely to prevent WebSocket connection crashes.</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>RECOMMENDED BASELINE.
-Saves 7.5% to 8.5% on streaming costs. Dynamic post-call summarization adds only $0.00096 USD per session (0.14% overhead), fully integrated in totals.</t>
+          <t>RECOMMENDED BASELINE FOR RAW SPEED.
+Saves 7.5% to 8.5% on streaming costs but cannot enforce a spoken clinical glossary. Post-call summary adds only $0.00096 USD (0.14% overhead).</t>
         </is>
       </c>
     </row>
@@ -648,18 +649,20 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Alternative translation approach where translation and pacing are guided via custom developer prompts.
-Post-call summary dynamically uses gemini-3.1-flash to align model families.</t>
+          <t>Alternative translation approach where translation and pacing are guided via custom system prompts.
+[PRO] FULLY supports custom system instructions and dynamic clinical glossary enforcement in synthesized spoken audio.
+Post-call summary dynamically uses gemini-3.1-flash.</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Requires custom pacing prompts and manual turn buffers, adding a +12.5% duration overhead to streaming audio outputs.</t>
+          <t>Requires custom pacing prompts and manual turn buffers, adding a +12.5% duration overhead to streaming audio outputs. System instruction includes the full clinical glossary, cached via Context Caching.</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Incurs higher streaming and text fees due to the pacing expansion and prompt instruction size. Dynamic post-call summarization is fully integrated.</t>
+          <t>RECOMMENDED FOR COMPLIANCE &amp; GLOSSARIES.
+Incurs slightly higher streaming fees due to the pacing expansion, but enforces medical terminology perfectly. Fully integrated with prompt caching.</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1100,7 @@
         </is>
       </c>
       <c r="B25" s="15" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="C25" s="15" t="n">
         <v>3000</v>
@@ -1107,7 +1110,7 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Static instructions + glossary context</t>
+          <t>Static instructions + glossary context (N/A for Approach A)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(cost-estimation): correct Gemini 3.5 live translate pricing and model name to gemini-3.1-flash-live-preview
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -18,16 +18,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$#,##0.000"/>
     <numFmt numFmtId="168" formatCode="$#,##0.00000"/>
     <numFmt numFmtId="169" formatCode="$#,##0.0000"/>
-    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="170" formatCode="$#,,##0.00"/>
+    <numFmt numFmtId="171" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +68,12 @@
     <font>
       <name val="Segoe UI"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Outfit"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="5">
@@ -129,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -162,6 +169,9 @@
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -178,10 +188,11 @@
     <xf numFmtId="166" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -644,7 +655,7 @@
         <is>
           <t>Approach B:
 Prompt-Driven Flash 3.1
-(gemini-3.1-flash)</t>
+(gemini-3.1-flash-live-preview)</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -732,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -740,6 +751,7 @@
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -775,6 +787,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -918,7 +931,7 @@
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>gemini-3.1-flash</t>
+          <t>gemini-3.1-flash-live-preview</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -929,6 +942,11 @@
       <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Unit</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Pricing Reference</t>
         </is>
       </c>
     </row>
@@ -939,7 +957,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>3</v>
@@ -952,6 +970,11 @@
           <t>per Million Tokens</t>
         </is>
       </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Studio Pricing</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
@@ -960,7 +983,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>12</v>
@@ -973,6 +996,11 @@
           <t>per Million Tokens</t>
         </is>
       </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Studio Pricing</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -981,17 +1009,22 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>0.75</v>
+        <v>3.5</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>0.75</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D18" s="15" t="n">
         <v>0.075</v>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
           <t>per Million Tokens</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Studio Pricing</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1035,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>4.5</v>
+        <v>21</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>4.5</v>
@@ -1015,6 +1048,11 @@
           <t>per Million Tokens</t>
         </is>
       </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Studio Pricing</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -1023,17 +1061,22 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>0.15</v>
       </c>
-      <c r="D20" s="14" t="n">
+      <c r="D20" s="15" t="n">
         <v>0.015</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
           <t>per Million Tokens</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Studio Pricing</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1087,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1</v>
@@ -1055,6 +1098,11 @@
       <c r="E21" s="9" t="inlineStr">
         <is>
           <t>per Million Tokens</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Studio Pricing</t>
         </is>
       </c>
     </row>
@@ -1099,13 +1147,13 @@
           <t>Prompt Cache Read Size (Tokens)</t>
         </is>
       </c>
-      <c r="B25" s="15" t="n">
+      <c r="B25" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="C25" s="15" t="n">
+      <c r="C25" s="16" t="n">
         <v>3000</v>
       </c>
-      <c r="D25" s="15" t="n">
+      <c r="D25" s="16" t="n">
         <v>3000</v>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -1120,15 +1168,15 @@
           <t>Prompt Cache Read Cost (USD)</t>
         </is>
       </c>
-      <c r="B26" s="16">
+      <c r="B26" s="17">
         <f>B25*(B20/1000000)</f>
         <v/>
       </c>
-      <c r="C26" s="16">
+      <c r="C26" s="17">
         <f>C25*(C20/1000000)</f>
         <v/>
       </c>
-      <c r="D26" s="16">
+      <c r="D26" s="17">
         <f>D25*(D20/1000000)</f>
         <v/>
       </c>
@@ -1144,15 +1192,15 @@
           <t>Audio Input Tokens per Session</t>
         </is>
       </c>
-      <c r="B27" s="15">
+      <c r="B27" s="16">
         <f>2*$B$6*60*250*$B$10*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="C27" s="15">
+      <c r="C27" s="16">
         <f>2*$B$6*60*250*$B$10*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="16">
         <f>2*$B$6*60*250*$B$10*(1+$B$11)</f>
         <v/>
       </c>
@@ -1192,15 +1240,15 @@
           <t>Spoken Dialogue Word Count (Est.)</t>
         </is>
       </c>
-      <c r="B29" s="15">
+      <c r="B29" s="16">
         <f>$B$6*$B$10*150</f>
         <v/>
       </c>
-      <c r="C29" s="15">
+      <c r="C29" s="16">
         <f>$B$6*$B$10*150</f>
         <v/>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="16">
         <f>$B$6*$B$10*150</f>
         <v/>
       </c>
@@ -1216,15 +1264,15 @@
           <t>Audio Output Pacing Duration (Sec)</t>
         </is>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="16">
         <f>(B29/2.5)*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="16">
         <f>(C29/2.5)*1.125*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="16">
         <f>(D29/2.5)*1.125*(1+$B$11)</f>
         <v/>
       </c>
@@ -1240,15 +1288,15 @@
           <t>Audio Output Tokens per Session</t>
         </is>
       </c>
-      <c r="B31" s="15">
+      <c r="B31" s="16">
         <f>B30*250</f>
         <v/>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="16">
         <f>C30*250</f>
         <v/>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="16">
         <f>D30*250</f>
         <v/>
       </c>
@@ -1288,15 +1336,15 @@
           <t>Transcription Text Output (Tokens)</t>
         </is>
       </c>
-      <c r="B33" s="15">
+      <c r="B33" s="16">
         <f>(B29*2.2)*1.33</f>
         <v/>
       </c>
-      <c r="C33" s="15">
+      <c r="C33" s="16">
         <f>(C29*2.2)*1.33</f>
         <v/>
       </c>
-      <c r="D33" s="15">
+      <c r="D33" s="16">
         <f>(D29*2.2)*1.33</f>
         <v/>
       </c>
@@ -1312,15 +1360,15 @@
           <t>Transcription Text Cost (USD)</t>
         </is>
       </c>
-      <c r="B34" s="17">
+      <c r="B34" s="18">
         <f>B33*(B19/1000000)</f>
         <v/>
       </c>
-      <c r="C34" s="17">
+      <c r="C34" s="18">
         <f>C33*(C19/1000000)</f>
         <v/>
       </c>
-      <c r="D34" s="17">
+      <c r="D34" s="18">
         <f>D33*(D19/1000000)</f>
         <v/>
       </c>
@@ -1336,15 +1384,15 @@
           <t>Post-Call Summary Input (Tokens)</t>
         </is>
       </c>
-      <c r="B35" s="15">
+      <c r="B35" s="16">
         <f>B33</f>
         <v/>
       </c>
-      <c r="C35" s="15">
+      <c r="C35" s="16">
         <f>C33</f>
         <v/>
       </c>
-      <c r="D35" s="15">
+      <c r="D35" s="16">
         <f>D33</f>
         <v/>
       </c>
@@ -1360,13 +1408,13 @@
           <t>Post-Call Summary Output (Tokens)</t>
         </is>
       </c>
-      <c r="B36" s="15" t="n">
+      <c r="B36" s="16" t="n">
         <v>1200</v>
       </c>
-      <c r="C36" s="15" t="n">
+      <c r="C36" s="16" t="n">
         <v>1200</v>
       </c>
-      <c r="D36" s="15" t="n">
+      <c r="D36" s="16" t="n">
         <v>1200</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
@@ -1381,15 +1429,15 @@
           <t>Post-Call Summary Cost (USD)</t>
         </is>
       </c>
-      <c r="B37" s="16">
+      <c r="B37" s="17">
         <f>(B35*(B18/1000000))+(B36*(B19/1000000))</f>
         <v/>
       </c>
-      <c r="C37" s="16">
+      <c r="C37" s="17">
         <f>(C35*(C18/1000000))+(C36*(C19/1000000))</f>
         <v/>
       </c>
-      <c r="D37" s="16">
+      <c r="D37" s="17">
         <f>(D35*(D18/1000000))+(D36*(D19/1000000))</f>
         <v/>
       </c>
@@ -1400,48 +1448,48 @@
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Total Session Cost (USD)</t>
         </is>
       </c>
-      <c r="B38" s="19">
+      <c r="B38" s="20">
         <f>B26+B28+B32+B34+B37</f>
         <v/>
       </c>
-      <c r="C38" s="19">
+      <c r="C38" s="20">
         <f>C26+C28+C32+C34+C37</f>
         <v/>
       </c>
-      <c r="D38" s="19">
+      <c r="D38" s="20">
         <f>D26+D28+D32+D34+D37</f>
         <v/>
       </c>
-      <c r="E38" s="18" t="inlineStr">
+      <c r="E38" s="19" t="inlineStr">
         <is>
           <t>Sum of all live streaming &amp; summary costs</t>
         </is>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="18" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>Total Session Cost (AUD)</t>
         </is>
       </c>
-      <c r="B39" s="19">
+      <c r="B39" s="20">
         <f>B38*$B$5</f>
         <v/>
       </c>
-      <c r="C39" s="19">
+      <c r="C39" s="20">
         <f>C38*$B$5</f>
         <v/>
       </c>
-      <c r="D39" s="19">
+      <c r="D39" s="20">
         <f>D38*$B$5</f>
         <v/>
       </c>
-      <c r="E39" s="18" t="inlineStr">
+      <c r="E39" s="19" t="inlineStr">
         <is>
           <t>USD Cost * Exchange Rate</t>
         </is>
@@ -1603,24 +1651,24 @@
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="18" t="inlineStr">
+      <c r="A48" s="19" t="inlineStr">
         <is>
           <t>Annual Cost (AUD)</t>
         </is>
       </c>
-      <c r="B48" s="19">
+      <c r="B48" s="20">
         <f>B47*$B$5</f>
         <v/>
       </c>
-      <c r="C48" s="19">
+      <c r="C48" s="20">
         <f>C47*$B$5</f>
         <v/>
       </c>
-      <c r="D48" s="19">
+      <c r="D48" s="20">
         <f>D47*$B$5</f>
         <v/>
       </c>
-      <c r="E48" s="18" t="inlineStr">
+      <c r="E48" s="19" t="inlineStr">
         <is>
           <t>Annual USD * Exchange Rate</t>
         </is>
@@ -1628,11 +1676,19 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A41:F41"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1643,7 +1699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1651,6 +1707,7 @@
     <col width="75" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -1674,7 +1731,7 @@
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -1684,8 +1741,13 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr"/>
+      <c r="D4" s="12" t="inlineStr"/>
+      <c r="E4" s="12" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Pricing Reference</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -1701,6 +1763,9 @@
           <t>Number of localized language dialects (Spanish, Arabic, Vietnamese, Hindi, Cantonese)</t>
         </is>
       </c>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -1716,6 +1781,9 @@
           <t>Number of standardized medical terms and phrases to translate for the session prompt context</t>
         </is>
       </c>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -1731,6 +1799,9 @@
           <t>Average input tokens per term (source word + translation instructions + context guidelines)</t>
         </is>
       </c>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1746,6 +1817,9 @@
           <t>Average output tokens per term (translated word + pronunciation phonetics + contextual note)</t>
         </is>
       </c>
+      <c r="D8" s="21" t="n"/>
+      <c r="E8" s="21" t="n"/>
+      <c r="F8" s="21" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
@@ -1753,12 +1827,19 @@
           <t>Model_Input_Rate_Per_Million</t>
         </is>
       </c>
-      <c r="B9" s="20" t="n">
+      <c r="B9" s="22" t="n">
         <v>1.25</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Unit cost rate of Gemini 1.5 Pro to generate high-quality clinical translations (USD / Million)</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Studio Pricing</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1849,19 @@
           <t>Model_Output_Rate_Per_Million</t>
         </is>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="22" t="n">
         <v>5</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Unit cost rate of Gemini 1.5 Pro to generate high-quality clinical translations (USD / Million)</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Studio Pricing</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1898,7 @@
           <t>Total Generation Input Tokens</t>
         </is>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <f>B6*B7*B5</f>
         <v/>
       </c>
@@ -1826,7 +1914,7 @@
           <t>Total Generation Output Tokens</t>
         </is>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <f>B6*B8*B5</f>
         <v/>
       </c>
@@ -1869,32 +1957,32 @@
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Total One-Time Cost (USD)</t>
         </is>
       </c>
-      <c r="B18" s="19">
+      <c r="B18" s="20">
         <f>B16+B17</f>
         <v/>
       </c>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>Sum of input and output translation costs</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Total One-Time Cost (AUD)</t>
         </is>
       </c>
-      <c r="B19" s="19">
+      <c r="B19" s="20">
         <f>B18*'Cost Calculator'!$B$5</f>
         <v/>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C19" s="19" t="inlineStr">
         <is>
           <t>Total USD Cost * Indicative Exchange Rate (Cost Calculator B5)</t>
         </is>
@@ -1933,7 +2021,7 @@
           <t>Annual_New_Term_Maintenance</t>
         </is>
       </c>
-      <c r="B23" s="15" t="n">
+      <c r="B23" s="16" t="n">
         <v>50</v>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -1948,7 +2036,7 @@
           <t>Maintenance Input Tokens (Annual)</t>
         </is>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <f>B23*B7*B5</f>
         <v/>
       </c>
@@ -1964,7 +2052,7 @@
           <t>Maintenance Output Tokens (Annual)</t>
         </is>
       </c>
-      <c r="B25" s="15">
+      <c r="B25" s="16">
         <f>B23*B8*B5</f>
         <v/>
       </c>
@@ -1975,32 +2063,32 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>Annual Maintenance Cost (USD)</t>
         </is>
       </c>
-      <c r="B26" s="19">
+      <c r="B26" s="20">
         <f>(B24*(B9/1000000))+(B25*(B10/1000000))</f>
         <v/>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C26" s="19" t="inlineStr">
         <is>
           <t>Annual (InputTokens*InputRate + OutputTokens*OutputRate) / 1,000,000</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Annual Maintenance Cost (AUD)</t>
         </is>
       </c>
-      <c r="B27" s="19">
+      <c r="B27" s="20">
         <f>B26*'Cost Calculator'!$B$5</f>
         <v/>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C27" s="19" t="inlineStr">
         <is>
           <t>Annual USD Cost * Indicative Exchange Rate (Cost Calculator B5)</t>
         </is>
@@ -2039,7 +2127,7 @@
           <t>Glossary Size in Session Cache (Tokens)</t>
         </is>
       </c>
-      <c r="B31" s="15">
+      <c r="B31" s="16">
         <f>B6*B8</f>
         <v/>
       </c>
@@ -2055,7 +2143,7 @@
           <t>Cache TTL / Inactivity Expiry (Hours)</t>
         </is>
       </c>
-      <c r="B32" s="21" t="n">
+      <c r="B32" s="23" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -2065,32 +2153,32 @@
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="18" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>Prompt Cache Storage Cost per Hour (USD)</t>
         </is>
       </c>
-      <c r="B33" s="22">
+      <c r="B33" s="24">
         <f>B31*('Cost Calculator'!B21/1000000)</f>
         <v/>
       </c>
-      <c r="C33" s="18" t="inlineStr">
+      <c r="C33" s="19" t="inlineStr">
         <is>
           <t>Total Cached Tokens * (Cost Calculator Cache Storage Rate B21 / 1,000,000)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>Prompt Cache Storage Cost per Hour (AUD)</t>
         </is>
       </c>
-      <c r="B34" s="22">
+      <c r="B34" s="24">
         <f>B33*'Cost Calculator'!$B$5</f>
         <v/>
       </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="C34" s="19" t="inlineStr">
         <is>
           <t>Cache Storage USD * Indicative Exchange Rate (Cost Calculator B5)</t>
         </is>
@@ -2114,11 +2202,15 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A12:F12"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(cost-estimation): model and document client-side VAD silence suppression in Excel and report
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -875,7 +875,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Estimated percentage per channel of active speech (microphones only stream when active)</t>
+          <t>Estimated percentage of session with active speech (Client-Side VAD assumes microphones only stream when speech is detected, suppressing silence)</t>
         </is>
       </c>
     </row>
@@ -1193,20 +1193,20 @@
         </is>
       </c>
       <c r="B27" s="16">
-        <f>2*$B$6*60*250*$B$10*(1+$B$11)</f>
+        <f>$B$6*60*250*$B$10*(1+$B$11)</f>
         <v/>
       </c>
       <c r="C27" s="16">
-        <f>2*$B$6*60*250*$B$10*(1+$B$11)</f>
+        <f>$B$6*60*250*$B$10*(1+$B$11)</f>
         <v/>
       </c>
       <c r="D27" s="16">
-        <f>2*$B$6*60*250*$B$10*(1+$B$11)</f>
+        <f>$B$6*60*250*$B$10*(1+$B$11)</f>
         <v/>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>2 connections * Duration in seconds * 250 tokens/sec * Duty Cycle * (1 + Overlap Overhead)</t>
+          <t>Active connection duration (Client VAD suppresses silence) * 250 tokens/sec * (1 + Overlap Overhead)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(cost-estimation): make total cost labels dynamic based on cell B6 average session length
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -746,7 +746,7 @@
   <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
@@ -1448,10 +1448,9 @@
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="19" t="inlineStr">
-        <is>
-          <t>Total Session Cost (USD)</t>
-        </is>
+      <c r="A38" s="19">
+        <f>"Total Session Cost (USD) - Per average session length: "&amp;B6&amp;" mins"</f>
+        <v/>
       </c>
       <c r="B38" s="20">
         <f>B26+B28+B32+B34+B37</f>
@@ -1472,10 +1471,9 @@
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>Total Session Cost (AUD)</t>
-        </is>
+      <c r="A39" s="19">
+        <f>"Total Session Cost (AUD) - Per average session length: "&amp;B6&amp;" mins"</f>
+        <v/>
       </c>
       <c r="B39" s="20">
         <f>B38*$B$5</f>

</xml_diff>

<commit_message>
fix(cost-estimation): add user-adjustable SOAP size in words and tokens, and link transcription expansion factor to cell B12
</commit_message>
<xml_diff>
--- a/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
+++ b/HealthDirect/live-translate/simultaneous/utils/cost_calculator_sheet.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -161,6 +161,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -897,20 +900,34 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
+          <t>Linguistic_Transcript_Expansion_Factor</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Estimated ratio of total transcribed words (spoken + translated) over original spoken words</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
           <t>Weekly_Session_Volume</t>
         </is>
       </c>
-      <c r="B12" s="10">
+      <c r="B13" s="10">
         <f>B7*B8/B9</f>
         <v/>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Dynamic weekly session volume: (Annual Volume * Target Rate) / Weeks Per Year</t>
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -924,17 +941,17 @@
           <t>Service/Item</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>gemini-3.5-live-translate-preview</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>gemini-3.1-flash-live-preview</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>gemini-2.5-flash</t>
         </is>
@@ -956,13 +973,13 @@
           <t>Audio Input</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n">
+      <c r="B16" s="14" t="n">
         <v>3.5</v>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="14" t="n">
         <v>3</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -970,7 +987,7 @@
           <t>per Million Tokens</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>Google AI Studio Pricing</t>
         </is>
@@ -982,13 +999,13 @@
           <t>Audio Output</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n">
+      <c r="B17" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="14" t="n">
         <v>12</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -996,7 +1013,7 @@
           <t>per Million Tokens</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>Google AI Studio Pricing</t>
         </is>
@@ -1008,13 +1025,13 @@
           <t>Text Input</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n">
+      <c r="B18" s="14" t="n">
         <v>3.5</v>
       </c>
-      <c r="C18" s="13" t="n">
+      <c r="C18" s="14" t="n">
         <v>0.75</v>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="16" t="n">
         <v>0.075</v>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -1022,7 +1039,7 @@
           <t>per Million Tokens</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="15" t="inlineStr">
         <is>
           <t>Google AI Studio Pricing</t>
         </is>
@@ -1034,13 +1051,13 @@
           <t>Text Output</t>
         </is>
       </c>
-      <c r="B19" s="13" t="n">
+      <c r="B19" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="C19" s="13" t="n">
+      <c r="C19" s="14" t="n">
         <v>4.5</v>
       </c>
-      <c r="D19" s="13" t="n">
+      <c r="D19" s="14" t="n">
         <v>0.3</v>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -1048,7 +1065,7 @@
           <t>per Million Tokens</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>Google AI Studio Pricing</t>
         </is>
@@ -1060,13 +1077,13 @@
           <t>Cached Read</t>
         </is>
       </c>
-      <c r="B20" s="13" t="n">
+      <c r="B20" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="13" t="n">
+      <c r="C20" s="14" t="n">
         <v>0.15</v>
       </c>
-      <c r="D20" s="15" t="n">
+      <c r="D20" s="16" t="n">
         <v>0.015</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -1074,7 +1091,7 @@
           <t>per Million Tokens</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>Google AI Studio Pricing</t>
         </is>
@@ -1086,13 +1103,13 @@
           <t>Cache Storage</t>
         </is>
       </c>
-      <c r="B21" s="13" t="n">
+      <c r="B21" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C21" s="13" t="n">
+      <c r="C21" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="13" t="n">
+      <c r="D21" s="14" t="n">
         <v>0.1</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -1100,7 +1117,7 @@
           <t>per Million Tokens</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>Google AI Studio Pricing</t>
         </is>
@@ -1120,17 +1137,17 @@
           <t>Metric/Calculation</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Approach A: Native 3.5</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>Approach B: 3.1 Flash Prompt-driven</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Approach C: 2.5 Flash Prompt-driven</t>
         </is>
@@ -1147,13 +1164,13 @@
           <t>Prompt Cache Read Size (Tokens)</t>
         </is>
       </c>
-      <c r="B25" s="16" t="n">
+      <c r="B25" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="C25" s="16" t="n">
+      <c r="C25" s="17" t="n">
         <v>3000</v>
       </c>
-      <c r="D25" s="16" t="n">
+      <c r="D25" s="17" t="n">
         <v>3000</v>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -1168,15 +1185,15 @@
           <t>Prompt Cache Read Cost (USD)</t>
         </is>
       </c>
-      <c r="B26" s="17">
+      <c r="B26" s="18">
         <f>B25*(B20/1000000)</f>
         <v/>
       </c>
-      <c r="C26" s="17">
+      <c r="C26" s="18">
         <f>C25*(C20/1000000)</f>
         <v/>
       </c>
-      <c r="D26" s="17">
+      <c r="D26" s="18">
         <f>D25*(D20/1000000)</f>
         <v/>
       </c>
@@ -1192,15 +1209,15 @@
           <t>Audio Input Tokens per Session</t>
         </is>
       </c>
-      <c r="B27" s="16">
+      <c r="B27" s="17">
         <f>$B$6*60*250*$B$10*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="C27" s="16">
+      <c r="C27" s="17">
         <f>$B$6*60*250*$B$10*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="D27" s="16">
+      <c r="D27" s="17">
         <f>$B$6*60*250*$B$10*(1+$B$11)</f>
         <v/>
       </c>
@@ -1216,15 +1233,15 @@
           <t>Audio Input Cost (USD)</t>
         </is>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="14">
         <f>B27*(B16/1000000)</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>C27*(C16/1000000)</f>
         <v/>
       </c>
-      <c r="D28" s="13">
+      <c r="D28" s="14">
         <f>D27*(D16/1000000)</f>
         <v/>
       </c>
@@ -1240,15 +1257,15 @@
           <t>Spoken Dialogue Word Count (Est.)</t>
         </is>
       </c>
-      <c r="B29" s="16">
+      <c r="B29" s="17">
         <f>$B$6*$B$10*150</f>
         <v/>
       </c>
-      <c r="C29" s="16">
+      <c r="C29" s="17">
         <f>$B$6*$B$10*150</f>
         <v/>
       </c>
-      <c r="D29" s="16">
+      <c r="D29" s="17">
         <f>$B$6*$B$10*150</f>
         <v/>
       </c>
@@ -1264,15 +1281,15 @@
           <t>Audio Output Pacing Duration (Sec)</t>
         </is>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="17">
         <f>(B29/2.5)*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="17">
         <f>(C29/2.5)*1.125*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="17">
         <f>(D29/2.5)*1.125*(1+$B$11)</f>
         <v/>
       </c>
@@ -1288,15 +1305,15 @@
           <t>Audio Output Tokens per Session</t>
         </is>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="17">
         <f>B30*250</f>
         <v/>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="17">
         <f>C30*250</f>
         <v/>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="17">
         <f>D30*250</f>
         <v/>
       </c>
@@ -1312,15 +1329,15 @@
           <t>Audio Output Cost (USD)</t>
         </is>
       </c>
-      <c r="B32" s="13">
+      <c r="B32" s="14">
         <f>B31*(B17/1000000)</f>
         <v/>
       </c>
-      <c r="C32" s="13">
+      <c r="C32" s="14">
         <f>C31*(C17/1000000)</f>
         <v/>
       </c>
-      <c r="D32" s="13">
+      <c r="D32" s="14">
         <f>D31*(D17/1000000)</f>
         <v/>
       </c>
@@ -1336,21 +1353,21 @@
           <t>Transcription Text Output (Tokens)</t>
         </is>
       </c>
-      <c r="B33" s="16">
-        <f>(B29*2.2)*1.33</f>
-        <v/>
-      </c>
-      <c r="C33" s="16">
-        <f>(C29*2.2)*1.33</f>
-        <v/>
-      </c>
-      <c r="D33" s="16">
-        <f>(D29*2.2)*1.33</f>
+      <c r="B33" s="17">
+        <f>(B29*$B$12)*1.33</f>
+        <v/>
+      </c>
+      <c r="C33" s="17">
+        <f>(C29*$B$12)*1.33</f>
+        <v/>
+      </c>
+      <c r="D33" s="17">
+        <f>(D29*$B$12)*1.33</f>
         <v/>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>(Spoken + Translated words) * 1.33 tokens/word</t>
+          <t>Spoken words * Linguistic Expansion (Cell B12) * 1.33 tokens/word</t>
         </is>
       </c>
     </row>
@@ -1360,15 +1377,15 @@
           <t>Transcription Text Cost (USD)</t>
         </is>
       </c>
-      <c r="B34" s="18">
+      <c r="B34" s="19">
         <f>B33*(B19/1000000)</f>
         <v/>
       </c>
-      <c r="C34" s="18">
+      <c r="C34" s="19">
         <f>C33*(C19/1000000)</f>
         <v/>
       </c>
-      <c r="D34" s="18">
+      <c r="D34" s="19">
         <f>D33*(D19/1000000)</f>
         <v/>
       </c>
@@ -1384,15 +1401,15 @@
           <t>Post-Call Summary Input (Tokens)</t>
         </is>
       </c>
-      <c r="B35" s="16">
+      <c r="B35" s="17">
         <f>B33</f>
         <v/>
       </c>
-      <c r="C35" s="16">
+      <c r="C35" s="17">
         <f>C33</f>
         <v/>
       </c>
-      <c r="D35" s="16">
+      <c r="D35" s="17">
         <f>D33</f>
         <v/>
       </c>
@@ -1405,95 +1422,118 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Post-Call Summary Output (Tokens)</t>
-        </is>
-      </c>
-      <c r="B36" s="16" t="n">
-        <v>1200</v>
-      </c>
-      <c r="C36" s="16" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D36" s="16" t="n">
-        <v>1200</v>
+          <t>Post-Call Summary Output (Words)</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="n">
+        <v>900</v>
+      </c>
+      <c r="C36" s="17" t="n">
+        <v>900</v>
+      </c>
+      <c r="D36" s="17" t="n">
+        <v>900</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Output size of the generated structured clinical SOAP note</t>
+          <t>Clinician SOAP note target length in words</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
+          <t>Post-Call Summary Output (Tokens)</t>
+        </is>
+      </c>
+      <c r="B37" s="17">
+        <f>B36*1.33</f>
+        <v/>
+      </c>
+      <c r="C37" s="17">
+        <f>C36*1.33</f>
+        <v/>
+      </c>
+      <c r="D37" s="17">
+        <f>D36*1.33</f>
+        <v/>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>Output size in tokens based on 1.33 tokens/word</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
           <t>Post-Call Summary Cost (USD)</t>
         </is>
       </c>
-      <c r="B37" s="17">
-        <f>(B35*(B18/1000000))+(B36*(B19/1000000))</f>
-        <v/>
-      </c>
-      <c r="C37" s="17">
-        <f>(C35*(C18/1000000))+(C36*(C19/1000000))</f>
-        <v/>
-      </c>
-      <c r="D37" s="17">
-        <f>(D35*(D18/1000000))+(D36*(D19/1000000))</f>
-        <v/>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="B38" s="18">
+        <f>(B35*(B18/1000000))+(B37*(B19/1000000))</f>
+        <v/>
+      </c>
+      <c r="C38" s="18">
+        <f>(C35*(C18/1000000))+(C37*(C19/1000000))</f>
+        <v/>
+      </c>
+      <c r="D38" s="18">
+        <f>(D35*(D18/1000000))+(D37*(D19/1000000))</f>
+        <v/>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>Summary (Input*InputRate + Output*OutputRate) / 1,000,000</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="19">
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="20">
         <f>"Total Session Cost (USD) - Per average session length: "&amp;B6&amp;" mins"</f>
         <v/>
       </c>
-      <c r="B38" s="20">
-        <f>B26+B28+B32+B34+B37</f>
-        <v/>
-      </c>
-      <c r="C38" s="20">
-        <f>C26+C28+C32+C34+C37</f>
-        <v/>
-      </c>
-      <c r="D38" s="20">
-        <f>D26+D28+D32+D34+D37</f>
-        <v/>
-      </c>
-      <c r="E38" s="19" t="inlineStr">
+      <c r="B39" s="21">
+        <f>B26+B28+B32+B34+B38</f>
+        <v/>
+      </c>
+      <c r="C39" s="21">
+        <f>C26+C28+C32+C34+C38</f>
+        <v/>
+      </c>
+      <c r="D39" s="21">
+        <f>D26+D28+D32+D34+D38</f>
+        <v/>
+      </c>
+      <c r="E39" s="20" t="inlineStr">
         <is>
           <t>Sum of all live streaming &amp; summary costs</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="19">
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="20">
         <f>"Total Session Cost (AUD) - Per average session length: "&amp;B6&amp;" mins"</f>
         <v/>
       </c>
-      <c r="B39" s="20">
-        <f>B38*$B$5</f>
-        <v/>
-      </c>
-      <c r="C39" s="20">
-        <f>C38*$B$5</f>
-        <v/>
-      </c>
-      <c r="D39" s="20">
-        <f>D38*$B$5</f>
-        <v/>
-      </c>
-      <c r="E39" s="19" t="inlineStr">
+      <c r="B40" s="21">
+        <f>B39*$B$5</f>
+        <v/>
+      </c>
+      <c r="C40" s="21">
+        <f>C39*$B$5</f>
+        <v/>
+      </c>
+      <c r="D40" s="21">
+        <f>D39*$B$5</f>
+        <v/>
+      </c>
+      <c r="E40" s="20" t="inlineStr">
         <is>
           <t>USD Cost * Exchange Rate</t>
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41" ht="24" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
@@ -1507,17 +1547,17 @@
           <t>Volume / Projections</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>Approach A: Native 3.5</t>
         </is>
       </c>
-      <c r="C42" s="12" t="inlineStr">
+      <c r="C42" s="13" t="inlineStr">
         <is>
           <t>Approach B: 3.1 Flash Prompt-driven</t>
         </is>
       </c>
-      <c r="D42" s="12" t="inlineStr">
+      <c r="D42" s="13" t="inlineStr">
         <is>
           <t>Approach C: 2.5 Flash Prompt-driven</t>
         </is>
@@ -1534,21 +1574,21 @@
           <t>Weekly Cost (USD)</t>
         </is>
       </c>
-      <c r="B43" s="13">
-        <f>B38*$B$12</f>
-        <v/>
-      </c>
-      <c r="C43" s="13">
-        <f>C38*$B$12</f>
-        <v/>
-      </c>
-      <c r="D43" s="13">
-        <f>D38*$B$12</f>
+      <c r="B43" s="14">
+        <f>B39*$B$13</f>
+        <v/>
+      </c>
+      <c r="C43" s="14">
+        <f>C39*$B$13</f>
+        <v/>
+      </c>
+      <c r="D43" s="14">
+        <f>D39*$B$13</f>
         <v/>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Sessions/Week * Session Cost (Row 38)</t>
+          <t>Sessions/Week * Session Cost (Row 39)</t>
         </is>
       </c>
     </row>
@@ -1558,15 +1598,15 @@
           <t>Weekly Cost (AUD)</t>
         </is>
       </c>
-      <c r="B44" s="13">
+      <c r="B44" s="14">
         <f>B43*$B$5</f>
         <v/>
       </c>
-      <c r="C44" s="13">
+      <c r="C44" s="14">
         <f>C43*$B$5</f>
         <v/>
       </c>
-      <c r="D44" s="13">
+      <c r="D44" s="14">
         <f>D43*$B$5</f>
         <v/>
       </c>
@@ -1582,15 +1622,15 @@
           <t>Monthly Cost (USD)</t>
         </is>
       </c>
-      <c r="B45" s="13">
+      <c r="B45" s="14">
         <f>B43*4.33</f>
         <v/>
       </c>
-      <c r="C45" s="13">
+      <c r="C45" s="14">
         <f>C43*4.33</f>
         <v/>
       </c>
-      <c r="D45" s="13">
+      <c r="D45" s="14">
         <f>D43*4.33</f>
         <v/>
       </c>
@@ -1606,15 +1646,15 @@
           <t>Monthly Cost (AUD)</t>
         </is>
       </c>
-      <c r="B46" s="13">
+      <c r="B46" s="14">
         <f>B45*$B$5</f>
         <v/>
       </c>
-      <c r="C46" s="13">
+      <c r="C46" s="14">
         <f>C45*$B$5</f>
         <v/>
       </c>
-      <c r="D46" s="13">
+      <c r="D46" s="14">
         <f>D45*$B$5</f>
         <v/>
       </c>
@@ -1630,15 +1670,15 @@
           <t>Annual Cost (USD)</t>
         </is>
       </c>
-      <c r="B47" s="13">
+      <c r="B47" s="14">
         <f>B43*52</f>
         <v/>
       </c>
-      <c r="C47" s="13">
+      <c r="C47" s="14">
         <f>C43*52</f>
         <v/>
       </c>
-      <c r="D47" s="13">
+      <c r="D47" s="14">
         <f>D43*52</f>
         <v/>
       </c>
@@ -1649,24 +1689,24 @@
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="19" t="inlineStr">
+      <c r="A48" s="20" t="inlineStr">
         <is>
           <t>Annual Cost (AUD)</t>
         </is>
       </c>
-      <c r="B48" s="20">
+      <c r="B48" s="21">
         <f>B47*$B$5</f>
         <v/>
       </c>
-      <c r="C48" s="20">
+      <c r="C48" s="21">
         <f>C47*$B$5</f>
         <v/>
       </c>
-      <c r="D48" s="20">
+      <c r="D48" s="21">
         <f>D47*$B$5</f>
         <v/>
       </c>
-      <c r="E48" s="19" t="inlineStr">
+      <c r="E48" s="20" t="inlineStr">
         <is>
           <t>Annual USD * Exchange Rate</t>
         </is>
@@ -1729,7 +1769,7 @@
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -1739,8 +1779,8 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="12" t="inlineStr"/>
+      <c r="D4" s="13" t="inlineStr"/>
+      <c r="E4" s="13" t="inlineStr"/>
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Pricing Reference</t>
@@ -1761,9 +1801,9 @@
           <t>Number of localized language dialects (Spanish, Arabic, Vietnamese, Hindi, Cantonese)</t>
         </is>
       </c>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="21" t="n"/>
-      <c r="F5" s="21" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="22" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -1779,9 +1819,9 @@
           <t>Number of standardized medical terms and phrases to translate for the session prompt context</t>
         </is>
       </c>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="21" t="n"/>
-      <c r="F6" s="21" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -1797,9 +1837,9 @@
           <t>Average input tokens per term (source word + translation instructions + context guidelines)</t>
         </is>
       </c>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="21" t="n"/>
-      <c r="F7" s="21" t="n"/>
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="22" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1815,9 +1855,9 @@
           <t>Average output tokens per term (translated word + pronunciation phonetics + contextual note)</t>
         </is>
       </c>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="21" t="n"/>
-      <c r="F8" s="21" t="n"/>
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="22" t="n"/>
+      <c r="F8" s="22" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
@@ -1825,7 +1865,7 @@
           <t>Model_Input_Rate_Per_Million</t>
         </is>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="23" t="n">
         <v>1.25</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1833,9 +1873,9 @@
           <t>Unit cost rate of Gemini 1.5 Pro to generate high-quality clinical translations (USD / Million)</t>
         </is>
       </c>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="21" t="n"/>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>Google AI Studio Pricing</t>
         </is>
@@ -1847,7 +1887,7 @@
           <t>Model_Output_Rate_Per_Million</t>
         </is>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="23" t="n">
         <v>5</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1855,9 +1895,9 @@
           <t>Unit cost rate of Gemini 1.5 Pro to generate high-quality clinical translations (USD / Million)</t>
         </is>
       </c>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>Google AI Studio Pricing</t>
         </is>
@@ -1877,7 +1917,7 @@
           <t>Calculation Metric</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -1887,8 +1927,8 @@
           <t>Formula Description</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr"/>
-      <c r="E13" s="12" t="inlineStr"/>
+      <c r="D13" s="13" t="inlineStr"/>
+      <c r="E13" s="13" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -1896,7 +1936,7 @@
           <t>Total Generation Input Tokens</t>
         </is>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="17">
         <f>B6*B7*B5</f>
         <v/>
       </c>
@@ -1912,7 +1952,7 @@
           <t>Total Generation Output Tokens</t>
         </is>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="17">
         <f>B6*B8*B5</f>
         <v/>
       </c>
@@ -1928,7 +1968,7 @@
           <t>Input Translation Cost (USD)</t>
         </is>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="14">
         <f>B14*(B9/1000000)</f>
         <v/>
       </c>
@@ -1944,7 +1984,7 @@
           <t>Output Translation Cost (USD)</t>
         </is>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="14">
         <f>B15*(B10/1000000)</f>
         <v/>
       </c>
@@ -1955,32 +1995,32 @@
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Total One-Time Cost (USD)</t>
         </is>
       </c>
-      <c r="B18" s="20">
+      <c r="B18" s="21">
         <f>B16+B17</f>
         <v/>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>Sum of input and output translation costs</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Total One-Time Cost (AUD)</t>
         </is>
       </c>
-      <c r="B19" s="20">
+      <c r="B19" s="21">
         <f>B18*'Cost Calculator'!$B$5</f>
         <v/>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>Total USD Cost * Indicative Exchange Rate (Cost Calculator B5)</t>
         </is>
@@ -2000,7 +2040,7 @@
           <t>Maintenance Metric</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -2010,8 +2050,8 @@
           <t>Formula Description</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="12" t="inlineStr"/>
+      <c r="D22" s="13" t="inlineStr"/>
+      <c r="E22" s="13" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -2019,7 +2059,7 @@
           <t>Annual_New_Term_Maintenance</t>
         </is>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B23" s="17" t="n">
         <v>50</v>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -2034,7 +2074,7 @@
           <t>Maintenance Input Tokens (Annual)</t>
         </is>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="17">
         <f>B23*B7*B5</f>
         <v/>
       </c>
@@ -2050,7 +2090,7 @@
           <t>Maintenance Output Tokens (Annual)</t>
         </is>
       </c>
-      <c r="B25" s="16">
+      <c r="B25" s="17">
         <f>B23*B8*B5</f>
         <v/>
       </c>
@@ -2061,32 +2101,32 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>Annual Maintenance Cost (USD)</t>
         </is>
       </c>
-      <c r="B26" s="20">
+      <c r="B26" s="21">
         <f>(B24*(B9/1000000))+(B25*(B10/1000000))</f>
         <v/>
       </c>
-      <c r="C26" s="19" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>Annual (InputTokens*InputRate + OutputTokens*OutputRate) / 1,000,000</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Annual Maintenance Cost (AUD)</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="21">
         <f>B26*'Cost Calculator'!$B$5</f>
         <v/>
       </c>
-      <c r="C27" s="19" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>Annual USD Cost * Indicative Exchange Rate (Cost Calculator B5)</t>
         </is>
@@ -2106,7 +2146,7 @@
           <t>Caching Parameter</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -2116,8 +2156,8 @@
           <t>Formula Description</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr"/>
-      <c r="E30" s="12" t="inlineStr"/>
+      <c r="D30" s="13" t="inlineStr"/>
+      <c r="E30" s="13" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
@@ -2125,7 +2165,7 @@
           <t>Glossary Size in Session Cache (Tokens)</t>
         </is>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="17">
         <f>B6*B8</f>
         <v/>
       </c>
@@ -2141,7 +2181,7 @@
           <t>Cache TTL / Inactivity Expiry (Hours)</t>
         </is>
       </c>
-      <c r="B32" s="23" t="n">
+      <c r="B32" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -2151,32 +2191,32 @@
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>Prompt Cache Storage Cost per Hour (USD)</t>
         </is>
       </c>
-      <c r="B33" s="24">
+      <c r="B33" s="25">
         <f>B31*('Cost Calculator'!B21/1000000)</f>
         <v/>
       </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>Total Cached Tokens * (Cost Calculator Cache Storage Rate B21 / 1,000,000)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="19" t="inlineStr">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>Prompt Cache Storage Cost per Hour (AUD)</t>
         </is>
       </c>
-      <c r="B34" s="24">
+      <c r="B34" s="25">
         <f>B33*'Cost Calculator'!$B$5</f>
         <v/>
       </c>
-      <c r="C34" s="19" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>Cache Storage USD * Indicative Exchange Rate (Cost Calculator B5)</t>
         </is>
@@ -2188,7 +2228,7 @@
           <t>Active Call Prompt Cache Read Savings (AUD)</t>
         </is>
       </c>
-      <c r="B35" s="13">
+      <c r="B35" s="14">
         <f>(3000-B31)*('Cost Calculator'!B20/1000000)*'Cost Calculator'!$B$5</f>
         <v/>
       </c>

</xml_diff>